<commit_message>
Script Updated: Add MDF Split
</commit_message>
<xml_diff>
--- a/inputs/Dashboard_Template.xlsx
+++ b/inputs/Dashboard_Template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wyze0-my.sharepoint.com/personal/tina_si_wyze_com/Documents/Microsoft Teams Chat Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{577818DA-AEBD-44AD-A16C-22500F65D2D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{946D5AD4-6A11-4D30-8485-251A9C7DD512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="880" yWindow="500" windowWidth="27640" windowHeight="15800" xr2:uid="{EF25A0A0-D905-8040-9105-6E088B9A13D9}"/>
   </bookViews>
@@ -78,7 +78,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A72" authorId="3" shapeId="0" xr:uid="{82AF0F11-C6B4-F04D-A9ED-3915416AF9D9}">
+    <comment ref="A86" authorId="3" shapeId="0" xr:uid="{82AF0F11-C6B4-F04D-A9ED-3915416AF9D9}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -86,7 +86,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A98" authorId="4" shapeId="0" xr:uid="{386011EC-DBE4-41A2-83DF-66AEF797BEDD}">
+    <comment ref="A112" authorId="4" shapeId="0" xr:uid="{386011EC-DBE4-41A2-83DF-66AEF797BEDD}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -94,7 +94,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A108" authorId="5" shapeId="0" xr:uid="{1AFEDADD-C365-E749-8232-528FAE26FA5F}">
+    <comment ref="A122" authorId="5" shapeId="0" xr:uid="{1AFEDADD-C365-E749-8232-528FAE26FA5F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -102,7 +102,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A134" authorId="6" shapeId="0" xr:uid="{7DA3C9F3-4C95-4438-8FD7-0EA0ADAF259C}">
+    <comment ref="A148" authorId="6" shapeId="0" xr:uid="{7DA3C9F3-4C95-4438-8FD7-0EA0ADAF259C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -110,7 +110,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A144" authorId="7" shapeId="0" xr:uid="{380AB180-B1D9-2D42-90D3-AB6531D1AE69}">
+    <comment ref="A158" authorId="7" shapeId="0" xr:uid="{380AB180-B1D9-2D42-90D3-AB6531D1AE69}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -118,7 +118,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A170" authorId="8" shapeId="0" xr:uid="{67A3F2EF-43BD-4596-8C9E-95EE0B936536}">
+    <comment ref="A184" authorId="8" shapeId="0" xr:uid="{67A3F2EF-43BD-4596-8C9E-95EE0B936536}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -126,7 +126,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A200" authorId="9" shapeId="0" xr:uid="{4D860FE9-95F1-44AC-8668-2173C60219B6}">
+    <comment ref="A214" authorId="9" shapeId="0" xr:uid="{4D860FE9-95F1-44AC-8668-2173C60219B6}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -134,7 +134,7 @@
     Monthly tracking following Finance data</t>
       </text>
     </comment>
-    <comment ref="A210" authorId="10" shapeId="0" xr:uid="{7D78CC43-3312-0244-804C-8514DA03F6E7}">
+    <comment ref="A224" authorId="10" shapeId="0" xr:uid="{7D78CC43-3312-0244-804C-8514DA03F6E7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -147,7 +147,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="48">
   <si>
     <t>Weeks starting</t>
   </si>
@@ -246,6 +246,12 @@
   </si>
   <si>
     <t>Total Marketing</t>
+  </si>
+  <si>
+    <t>Non-MDF</t>
+  </si>
+  <si>
+    <t>MDF</t>
   </si>
   <si>
     <t>Ads - On-site</t>
@@ -898,28 +904,28 @@
   <threadedComment ref="A56" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{634ACAA1-0E94-4376-ACB7-71D8813F2AF1}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A72" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{82AF0F11-C6B4-F04D-A9ED-3915416AF9D9}">
+  <threadedComment ref="A86" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{82AF0F11-C6B4-F04D-A9ED-3915416AF9D9}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A98" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{386011EC-DBE4-41A2-83DF-66AEF797BEDD}">
+  <threadedComment ref="A112" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{386011EC-DBE4-41A2-83DF-66AEF797BEDD}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A108" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{1AFEDADD-C365-E749-8232-528FAE26FA5F}">
+  <threadedComment ref="A122" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{1AFEDADD-C365-E749-8232-528FAE26FA5F}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A134" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{7DA3C9F3-4C95-4438-8FD7-0EA0ADAF259C}">
+  <threadedComment ref="A148" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{7DA3C9F3-4C95-4438-8FD7-0EA0ADAF259C}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A144" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{380AB180-B1D9-2D42-90D3-AB6531D1AE69}">
+  <threadedComment ref="A158" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{380AB180-B1D9-2D42-90D3-AB6531D1AE69}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A170" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{67A3F2EF-43BD-4596-8C9E-95EE0B936536}">
+  <threadedComment ref="A184" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{67A3F2EF-43BD-4596-8C9E-95EE0B936536}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A200" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{4D860FE9-95F1-44AC-8668-2173C60219B6}">
+  <threadedComment ref="A214" dT="2026-05-15T18:20:35.28" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{4D860FE9-95F1-44AC-8668-2173C60219B6}">
     <text>Monthly tracking following Finance data</text>
   </threadedComment>
-  <threadedComment ref="A210" dT="2026-05-15T18:24:20.75" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{7D78CC43-3312-0244-804C-8514DA03F6E7}">
+  <threadedComment ref="A224" dT="2026-05-15T18:24:20.75" personId="{19D00E75-0F05-0A4F-A966-774F535A6025}" id="{7D78CC43-3312-0244-804C-8514DA03F6E7}">
     <text>Monthly tracking following finance data</text>
   </threadedComment>
 </ThreadedComments>
@@ -927,7 +933,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE93501D-7553-084B-9556-DB9CF7693BED}">
-  <dimension ref="A1:CI248"/>
+  <dimension ref="A1:CI262"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
     <col min="1" max="1" width="34.25" bestFit="1" customWidth="1"/>
@@ -1669,376 +1675,377 @@
       <c r="A63" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B63" s="1" t="s">
-        <v>26</v>
-      </c>
+      <c r="B63" s="1"/>
       <c r="C63" s="1"/>
       <c r="D63" s="23" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="15.75">
-      <c r="B64" s="9" t="s">
+      <c r="A64" s="1"/>
+      <c r="B64" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C64" s="1"/>
+      <c r="D64" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" ht="15.75">
+      <c r="A65" s="50">
+        <f>SUM(E65:BE65)</f>
+        <v>0</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" ht="15.75">
+      <c r="B66" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D66" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" ht="15.75">
+      <c r="B67" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D67" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="15.75">
+      <c r="B68" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D68" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" ht="15.75"/>
+    <row r="70" spans="1:4" ht="15.75">
+      <c r="A70" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D64" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="65" spans="1:57" ht="15.75"/>
-    <row r="66" spans="1:57" ht="15.75">
-      <c r="A66" s="1" t="s">
+      <c r="B70" s="1"/>
+      <c r="C70" s="1"/>
+      <c r="D70" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" ht="15.75">
+      <c r="A71" s="1"/>
+      <c r="B71" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C71" s="1"/>
+      <c r="D71" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" ht="15.75">
+      <c r="A72" s="50">
+        <f>SUM(E72:BE72)</f>
+        <v>0</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="D72" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" ht="15.75">
+      <c r="B73" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D73" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" ht="15.75">
+      <c r="B74" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D74" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" ht="15.75">
+      <c r="B75" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D75" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="15.75"/>
+    <row r="77" spans="1:4" ht="15.75">
+      <c r="A77" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B66" s="1" t="s">
+      <c r="B77" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C66" s="1"/>
-      <c r="D66" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:57" ht="15.75">
-      <c r="B67" s="9" t="s">
+      <c r="C77" s="1"/>
+      <c r="D77" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="15.75">
+      <c r="B78" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="D67" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="68" spans="1:57" ht="15.75"/>
-    <row r="69" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A69" s="1" t="s">
+      <c r="D78" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="15.75"/>
+    <row r="80" spans="1:4" ht="15.75">
+      <c r="A80" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B69" s="1" t="s">
+      <c r="B80" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D69" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:57" ht="15.75">
-      <c r="B70" s="9" t="s">
+      <c r="C80" s="1"/>
+      <c r="D80" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="81" spans="1:57" ht="15.75">
+      <c r="B81" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D81" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="82" spans="1:57" ht="15.75"/>
+    <row r="83" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A83" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D83" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:57" ht="15.75">
+      <c r="B84" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D70" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:57" ht="15.75"/>
-    <row r="72" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A72" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B72" s="1" t="s">
+      <c r="D84" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="85" spans="1:57" ht="15.75"/>
+    <row r="86" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A86" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B86" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D72" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E72"/>
-      <c r="F72"/>
-      <c r="G72"/>
-      <c r="H72"/>
-      <c r="I72"/>
-      <c r="J72"/>
-      <c r="K72"/>
-      <c r="L72"/>
-      <c r="M72"/>
-      <c r="N72"/>
-      <c r="O72"/>
-      <c r="P72"/>
-      <c r="Q72"/>
-      <c r="R72"/>
-      <c r="S72"/>
-      <c r="T72"/>
-      <c r="U72"/>
-      <c r="V72"/>
-      <c r="W72"/>
-      <c r="X72"/>
-      <c r="Y72"/>
-      <c r="Z72"/>
-      <c r="AA72"/>
-      <c r="AB72"/>
-      <c r="AC72"/>
-      <c r="AD72"/>
-      <c r="AE72"/>
-      <c r="AF72"/>
-      <c r="AG72"/>
-      <c r="AH72"/>
-      <c r="AI72"/>
-      <c r="AJ72"/>
-      <c r="AK72"/>
-      <c r="AL72"/>
-      <c r="AM72"/>
-      <c r="AN72"/>
-      <c r="AO72"/>
-      <c r="AP72"/>
-      <c r="AQ72"/>
-      <c r="AR72"/>
-      <c r="AS72"/>
-      <c r="AT72"/>
-      <c r="AU72"/>
-      <c r="AV72"/>
-      <c r="AW72"/>
-      <c r="AX72"/>
-      <c r="AY72"/>
-      <c r="AZ72"/>
-      <c r="BA72"/>
-      <c r="BB72"/>
-      <c r="BC72"/>
-      <c r="BD72"/>
-      <c r="BE72"/>
-    </row>
-    <row r="73" spans="1:57" ht="15.75">
-      <c r="B73" s="9" t="s">
+      <c r="D86" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E86"/>
+      <c r="F86"/>
+      <c r="G86"/>
+      <c r="H86"/>
+      <c r="I86"/>
+      <c r="J86"/>
+      <c r="K86"/>
+      <c r="L86"/>
+      <c r="M86"/>
+      <c r="N86"/>
+      <c r="O86"/>
+      <c r="P86"/>
+      <c r="Q86"/>
+      <c r="R86"/>
+      <c r="S86"/>
+      <c r="T86"/>
+      <c r="U86"/>
+      <c r="V86"/>
+      <c r="W86"/>
+      <c r="X86"/>
+      <c r="Y86"/>
+      <c r="Z86"/>
+      <c r="AA86"/>
+      <c r="AB86"/>
+      <c r="AC86"/>
+      <c r="AD86"/>
+      <c r="AE86"/>
+      <c r="AF86"/>
+      <c r="AG86"/>
+      <c r="AH86"/>
+      <c r="AI86"/>
+      <c r="AJ86"/>
+      <c r="AK86"/>
+      <c r="AL86"/>
+      <c r="AM86"/>
+      <c r="AN86"/>
+      <c r="AO86"/>
+      <c r="AP86"/>
+      <c r="AQ86"/>
+      <c r="AR86"/>
+      <c r="AS86"/>
+      <c r="AT86"/>
+      <c r="AU86"/>
+      <c r="AV86"/>
+      <c r="AW86"/>
+      <c r="AX86"/>
+      <c r="AY86"/>
+      <c r="AZ86"/>
+      <c r="BA86"/>
+      <c r="BB86"/>
+      <c r="BC86"/>
+      <c r="BD86"/>
+      <c r="BE86"/>
+    </row>
+    <row r="87" spans="1:57" ht="15.75">
+      <c r="B87" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D73" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="74" spans="1:57" ht="15.75"/>
-    <row r="75" spans="1:57" ht="15.75"/>
-    <row r="76" spans="1:57" s="25" customFormat="1" ht="15.75">
-      <c r="A76" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="D76" s="26"/>
-    </row>
-    <row r="77" spans="1:57" ht="15.75">
-      <c r="A77" s="1" t="s">
+      <c r="D87" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="88" spans="1:57" ht="15.75"/>
+    <row r="89" spans="1:57" ht="15.75"/>
+    <row r="90" spans="1:57" s="25" customFormat="1" ht="15.75">
+      <c r="A90" s="24" t="s">
+        <v>41</v>
+      </c>
+      <c r="D90" s="26"/>
+    </row>
+    <row r="91" spans="1:57" ht="15.75">
+      <c r="A91" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D77" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="78" spans="1:57" s="4" customFormat="1" ht="15.75">
-      <c r="A78" s="3"/>
-      <c r="B78" s="4" t="s">
+      <c r="D91" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:57" s="4" customFormat="1" ht="15.75">
+      <c r="A92" s="3"/>
+      <c r="B92" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D78" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="79" spans="1:57" s="7" customFormat="1" ht="15.75">
-      <c r="B79" s="7" t="s">
+      <c r="D92" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="93" spans="1:57" s="7" customFormat="1" ht="15.75">
+      <c r="B93" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D79" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="80" spans="1:57" s="7" customFormat="1" ht="15.75">
-      <c r="B80" s="7" t="s">
+      <c r="D93" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="94" spans="1:57" s="7" customFormat="1" ht="15.75">
+      <c r="B94" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C80" s="15"/>
-      <c r="D80" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" s="9" customFormat="1" ht="15.75">
-      <c r="A81" s="50">
-        <f>SUM(E81:BE81)</f>
+      <c r="C94" s="15"/>
+      <c r="D94" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="95" spans="1:57" s="9" customFormat="1" ht="15.75">
+      <c r="A95" s="50">
+        <f>SUM(E95:BE95)</f>
         <v>0</v>
       </c>
-      <c r="B81" s="9" t="s">
+      <c r="B95" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D81" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="15.75"/>
-    <row r="83" spans="1:4" ht="15.75">
-      <c r="A83" s="1" t="s">
+      <c r="D95" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="96" spans="1:57" ht="15.75"/>
+    <row r="97" spans="1:4" ht="15.75">
+      <c r="A97" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D83" s="23" t="s">
+      <c r="D97" s="23" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="84" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A84" s="3"/>
-      <c r="B84" s="4" t="s">
+    <row r="98" spans="1:4" s="4" customFormat="1" ht="15.75">
+      <c r="A98" s="3"/>
+      <c r="B98" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D84" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A85" s="14"/>
-      <c r="B85" s="15" t="s">
+      <c r="D98" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A99" s="14"/>
+      <c r="B99" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D85" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A86" s="14"/>
-      <c r="B86" s="7" t="s">
+      <c r="D99" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A100" s="14"/>
+      <c r="B100" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D86" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" s="12" customFormat="1" ht="15.75">
-      <c r="A87" s="50">
-        <f>SUM(E87:BE87)</f>
+      <c r="D100" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" s="12" customFormat="1" ht="15.75">
+      <c r="A101" s="50">
+        <f>SUM(E101:BE101)</f>
         <v>0</v>
       </c>
-      <c r="B87" s="12" t="s">
+      <c r="B101" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D87" s="13" t="s">
+      <c r="D101" s="13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="15.75">
-      <c r="B88" t="s">
+    <row r="102" spans="1:4" ht="15.75">
+      <c r="B102" t="s">
         <v>15</v>
       </c>
-      <c r="C88" s="11" t="s">
+      <c r="C102" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D88" s="6" t="s">
+      <c r="D102" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="15.75">
-      <c r="C89" s="11" t="s">
+    <row r="103" spans="1:4" ht="15.75">
+      <c r="C103" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D89" s="6" t="s">
+      <c r="D103" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="90" spans="1:4" ht="15.75">
-      <c r="C90" s="6"/>
-    </row>
-    <row r="91" spans="1:4" s="1" customFormat="1" ht="15.75">
-      <c r="A91" s="1" t="s">
+    <row r="104" spans="1:4" ht="15.75">
+      <c r="C104" s="6"/>
+    </row>
+    <row r="105" spans="1:4" s="1" customFormat="1" ht="15.75">
+      <c r="A105" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B91" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D91" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" s="1" customFormat="1" ht="15.75">
-      <c r="B92" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="D92" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" s="9" customFormat="1" ht="15.75">
-      <c r="A93" s="50">
-        <f>SUM(E93:BE93)</f>
-        <v>0</v>
-      </c>
-      <c r="B93" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D93" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="15.75">
-      <c r="B94" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D94" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="15.75">
-      <c r="B95" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D95" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="15.75">
-      <c r="B96" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D96" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="97" spans="1:60" ht="15.75"/>
-    <row r="98" spans="1:60" ht="15.75">
-      <c r="A98" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B98" s="1"/>
-      <c r="C98" s="1"/>
-      <c r="D98" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="99" spans="1:60" ht="15.75">
-      <c r="A99" s="1"/>
-      <c r="B99" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="C99" s="1"/>
-      <c r="D99" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="100" spans="1:60" ht="15.75">
-      <c r="A100" s="50">
-        <f>SUM(E100:BE100)</f>
-        <v>0</v>
-      </c>
-      <c r="B100" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D100" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="101" spans="1:60" ht="15.75">
-      <c r="B101" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D101" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="102" spans="1:60" ht="15.75">
-      <c r="B102" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D102" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="103" spans="1:60" ht="15.75">
-      <c r="B103" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D103" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="104" spans="1:60" ht="15.75"/>
-    <row r="105" spans="1:60" s="1" customFormat="1" ht="15.75">
-      <c r="A105" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>26</v>
@@ -2047,329 +2054,329 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:60" ht="15.75">
-      <c r="B106" s="9" t="s">
+    <row r="106" spans="1:4" s="1" customFormat="1" ht="15.75">
+      <c r="B106" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="D106" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" s="9" customFormat="1" ht="15.75">
+      <c r="A107" s="50">
+        <f>SUM(E107:BE107)</f>
+        <v>0</v>
+      </c>
+      <c r="B107" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C106" s="9"/>
-      <c r="D106" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="107" spans="1:60" ht="15.75"/>
-    <row r="108" spans="1:60" s="1" customFormat="1" ht="15.75">
-      <c r="A108" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D108" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E108"/>
-      <c r="F108"/>
-      <c r="G108"/>
-      <c r="H108"/>
-      <c r="I108"/>
-      <c r="J108"/>
-      <c r="K108"/>
-      <c r="L108"/>
-      <c r="M108"/>
-      <c r="N108"/>
-      <c r="O108"/>
-      <c r="P108"/>
-      <c r="Q108"/>
-      <c r="R108"/>
-      <c r="S108"/>
-      <c r="T108"/>
-      <c r="U108"/>
-      <c r="V108"/>
-      <c r="W108"/>
-      <c r="X108"/>
-      <c r="Y108"/>
-      <c r="Z108"/>
-      <c r="AA108"/>
-      <c r="AB108"/>
-      <c r="AC108"/>
-      <c r="AD108"/>
-      <c r="AE108"/>
-      <c r="AF108"/>
-      <c r="AG108"/>
-      <c r="AH108"/>
-      <c r="AI108"/>
-      <c r="AJ108"/>
-      <c r="AK108"/>
-      <c r="AL108"/>
-      <c r="AM108"/>
-      <c r="AN108"/>
-      <c r="AO108"/>
-      <c r="AP108"/>
-      <c r="AQ108"/>
-      <c r="AR108"/>
-      <c r="AS108"/>
-      <c r="AT108"/>
-      <c r="AU108"/>
-      <c r="AV108"/>
-      <c r="AW108"/>
-      <c r="AX108"/>
-      <c r="AY108"/>
-      <c r="AZ108"/>
-      <c r="BA108"/>
-      <c r="BB108"/>
-      <c r="BC108"/>
-      <c r="BD108"/>
-      <c r="BE108"/>
-      <c r="BF108"/>
-      <c r="BG108"/>
-      <c r="BH108"/>
-    </row>
-    <row r="109" spans="1:60" ht="15.75">
-      <c r="B109" s="9" t="s">
+      <c r="D107" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" ht="15.75">
+      <c r="B108" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D108" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="15.75">
+      <c r="B109" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D109" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="15.75">
+      <c r="B110" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D110" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" ht="15.75"/>
+    <row r="112" spans="1:4" ht="15.75">
+      <c r="A112" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B112" s="1"/>
+      <c r="C112" s="1"/>
+      <c r="D112" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="113" spans="1:60" ht="15.75">
+      <c r="A113" s="1"/>
+      <c r="B113" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C113" s="1"/>
+      <c r="D113" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="114" spans="1:60" ht="15.75">
+      <c r="A114" s="50">
+        <f>SUM(E114:BE114)</f>
+        <v>0</v>
+      </c>
+      <c r="B114" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C109" s="9"/>
-      <c r="D109" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="110" spans="1:60" ht="15.75"/>
-    <row r="111" spans="1:60" ht="15.75"/>
-    <row r="112" spans="1:60" s="28" customFormat="1" ht="15.75">
-      <c r="A112" s="27" t="s">
+      <c r="D114" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="115" spans="1:60" ht="15.75">
+      <c r="B115" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D115" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="116" spans="1:60" ht="15.75">
+      <c r="B116" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D116" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="117" spans="1:60" ht="15.75">
+      <c r="B117" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D117" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="118" spans="1:60" ht="15.75"/>
+    <row r="119" spans="1:60" s="1" customFormat="1" ht="15.75">
+      <c r="A119" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D112" s="29"/>
-    </row>
-    <row r="113" spans="1:4" ht="15.75">
-      <c r="A113" s="1" t="s">
+      <c r="B119" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D119" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="120" spans="1:60" ht="15.75">
+      <c r="B120" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C120" s="9"/>
+      <c r="D120" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="121" spans="1:60" ht="15.75"/>
+    <row r="122" spans="1:60" s="1" customFormat="1" ht="15.75">
+      <c r="A122" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D122" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E122"/>
+      <c r="F122"/>
+      <c r="G122"/>
+      <c r="H122"/>
+      <c r="I122"/>
+      <c r="J122"/>
+      <c r="K122"/>
+      <c r="L122"/>
+      <c r="M122"/>
+      <c r="N122"/>
+      <c r="O122"/>
+      <c r="P122"/>
+      <c r="Q122"/>
+      <c r="R122"/>
+      <c r="S122"/>
+      <c r="T122"/>
+      <c r="U122"/>
+      <c r="V122"/>
+      <c r="W122"/>
+      <c r="X122"/>
+      <c r="Y122"/>
+      <c r="Z122"/>
+      <c r="AA122"/>
+      <c r="AB122"/>
+      <c r="AC122"/>
+      <c r="AD122"/>
+      <c r="AE122"/>
+      <c r="AF122"/>
+      <c r="AG122"/>
+      <c r="AH122"/>
+      <c r="AI122"/>
+      <c r="AJ122"/>
+      <c r="AK122"/>
+      <c r="AL122"/>
+      <c r="AM122"/>
+      <c r="AN122"/>
+      <c r="AO122"/>
+      <c r="AP122"/>
+      <c r="AQ122"/>
+      <c r="AR122"/>
+      <c r="AS122"/>
+      <c r="AT122"/>
+      <c r="AU122"/>
+      <c r="AV122"/>
+      <c r="AW122"/>
+      <c r="AX122"/>
+      <c r="AY122"/>
+      <c r="AZ122"/>
+      <c r="BA122"/>
+      <c r="BB122"/>
+      <c r="BC122"/>
+      <c r="BD122"/>
+      <c r="BE122"/>
+      <c r="BF122"/>
+      <c r="BG122"/>
+      <c r="BH122"/>
+    </row>
+    <row r="123" spans="1:60" ht="15.75">
+      <c r="B123" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C123" s="9"/>
+      <c r="D123" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="124" spans="1:60" ht="15.75"/>
+    <row r="125" spans="1:60" ht="15.75"/>
+    <row r="126" spans="1:60" s="28" customFormat="1" ht="15.75">
+      <c r="A126" s="27" t="s">
+        <v>44</v>
+      </c>
+      <c r="D126" s="29"/>
+    </row>
+    <row r="127" spans="1:60" ht="15.75">
+      <c r="A127" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D113" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="114" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A114" s="3"/>
-      <c r="B114" s="4" t="s">
+      <c r="D127" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="128" spans="1:60" s="4" customFormat="1" ht="15.75">
+      <c r="A128" s="3"/>
+      <c r="B128" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D114" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="115" spans="1:4" s="7" customFormat="1" ht="15.75">
-      <c r="B115" s="7" t="s">
+      <c r="D128" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" s="7" customFormat="1" ht="15.75">
+      <c r="B129" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D115" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="116" spans="1:4" s="7" customFormat="1" ht="15.75">
-      <c r="B116" s="7" t="s">
+      <c r="D129" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" s="7" customFormat="1" ht="15.75">
+      <c r="B130" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C116" s="15"/>
-      <c r="D116" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" s="9" customFormat="1" ht="15.75">
-      <c r="A117" s="50">
-        <f>SUM(E117:BE117)</f>
+      <c r="C130" s="15"/>
+      <c r="D130" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4" s="9" customFormat="1" ht="15.75">
+      <c r="A131" s="50">
+        <f>SUM(E131:BE131)</f>
         <v>0</v>
       </c>
-      <c r="B117" s="9" t="s">
+      <c r="B131" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D117" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="15.75"/>
-    <row r="119" spans="1:4" ht="15.75">
-      <c r="A119" s="1" t="s">
+      <c r="D131" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4" ht="15.75"/>
+    <row r="133" spans="1:4" ht="15.75">
+      <c r="A133" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D119" s="23" t="s">
+      <c r="D133" s="23" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="120" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A120" s="3"/>
-      <c r="B120" s="4" t="s">
+    <row r="134" spans="1:4" s="4" customFormat="1" ht="15.75">
+      <c r="A134" s="3"/>
+      <c r="B134" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D120" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="121" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A121" s="14"/>
-      <c r="B121" s="15" t="s">
+      <c r="D134" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A135" s="14"/>
+      <c r="B135" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D121" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="122" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A122" s="50"/>
-      <c r="B122" s="7" t="s">
+      <c r="D135" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A136" s="50"/>
+      <c r="B136" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D122" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="123" spans="1:4" s="12" customFormat="1" ht="15.75">
-      <c r="A123" s="50">
-        <f>SUM(E123:BE123)</f>
+      <c r="D136" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4" s="12" customFormat="1" ht="15.75">
+      <c r="A137" s="50">
+        <f>SUM(E137:BE137)</f>
         <v>0</v>
       </c>
-      <c r="B123" s="12" t="s">
+      <c r="B137" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D123" s="13" t="s">
+      <c r="D137" s="13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="15.75">
-      <c r="B124" t="s">
+    <row r="138" spans="1:4" ht="15.75">
+      <c r="B138" t="s">
         <v>15</v>
       </c>
-      <c r="C124" s="11" t="s">
+      <c r="C138" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D124" s="6" t="s">
+      <c r="D138" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="15.75">
-      <c r="C125" s="11" t="s">
+    <row r="139" spans="1:4" ht="15.75">
+      <c r="C139" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D125" s="6" t="s">
+      <c r="D139" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="15.75">
-      <c r="C126" s="6"/>
-    </row>
-    <row r="127" spans="1:4" s="1" customFormat="1" ht="15.75">
-      <c r="A127" s="1" t="s">
+    <row r="140" spans="1:4" ht="15.75">
+      <c r="C140" s="6"/>
+    </row>
+    <row r="141" spans="1:4" s="1" customFormat="1" ht="15.75">
+      <c r="A141" s="1" t="s">
         <v>25</v>
-      </c>
-      <c r="B127" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D127" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" s="1" customFormat="1" ht="15.75">
-      <c r="B128" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="D128" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="129" spans="1:57" s="9" customFormat="1" ht="15.75">
-      <c r="A129" s="50">
-        <f>SUM(E129:BE129)</f>
-        <v>0</v>
-      </c>
-      <c r="B129" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D129" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="130" spans="1:57" ht="15.75">
-      <c r="B130" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D130" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="131" spans="1:57" ht="15.75">
-      <c r="B131" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D131" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="132" spans="1:57" ht="15.75">
-      <c r="B132" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D132" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="133" spans="1:57" ht="15.75"/>
-    <row r="134" spans="1:57" ht="15.75">
-      <c r="A134" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B134" s="1"/>
-      <c r="C134" s="1"/>
-      <c r="D134" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="135" spans="1:57" ht="15.75">
-      <c r="A135" s="1"/>
-      <c r="B135" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="C135" s="1"/>
-      <c r="D135" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="136" spans="1:57" ht="15.75">
-      <c r="A136" s="50">
-        <f>SUM(E136:BE136)</f>
-        <v>0</v>
-      </c>
-      <c r="B136" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D136" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="137" spans="1:57" ht="15.75">
-      <c r="B137" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D137" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="138" spans="1:57" ht="15.75">
-      <c r="B138" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D138" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="139" spans="1:57" ht="15.75">
-      <c r="B139" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D139" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="140" spans="1:57" ht="15.75"/>
-    <row r="141" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A141" s="1" t="s">
-        <v>40</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>26</v>
@@ -2378,667 +2385,666 @@
         <v>3</v>
       </c>
     </row>
-    <row r="142" spans="1:57" ht="15.75">
-      <c r="A142" s="50"/>
-      <c r="B142" s="9" t="s">
+    <row r="142" spans="1:4" s="1" customFormat="1" ht="15.75">
+      <c r="B142" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="D142" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4" s="9" customFormat="1" ht="15.75">
+      <c r="A143" s="50">
+        <f>SUM(E143:BE143)</f>
+        <v>0</v>
+      </c>
+      <c r="B143" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C142" s="9"/>
-      <c r="D142" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="143" spans="1:57" ht="15.75"/>
-    <row r="144" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A144" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D144" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E144"/>
-      <c r="F144"/>
-      <c r="G144"/>
-      <c r="H144"/>
-      <c r="I144"/>
-      <c r="J144"/>
-      <c r="K144"/>
-      <c r="L144"/>
-      <c r="M144"/>
-      <c r="N144"/>
-      <c r="O144"/>
-      <c r="P144"/>
-      <c r="Q144"/>
-      <c r="R144"/>
-      <c r="S144"/>
-      <c r="T144"/>
-      <c r="U144"/>
-      <c r="V144"/>
-      <c r="W144"/>
-      <c r="X144"/>
-      <c r="Y144"/>
-      <c r="Z144"/>
-      <c r="AA144"/>
-      <c r="AB144"/>
-      <c r="AC144"/>
-      <c r="AD144"/>
-      <c r="AE144"/>
-      <c r="AF144"/>
-      <c r="AG144"/>
-      <c r="AH144"/>
-      <c r="AI144"/>
-      <c r="AJ144"/>
-      <c r="AK144"/>
-      <c r="AL144"/>
-      <c r="AM144"/>
-      <c r="AN144"/>
-      <c r="AO144"/>
-      <c r="AP144"/>
-      <c r="AQ144"/>
-      <c r="AR144"/>
-      <c r="AS144"/>
-      <c r="AT144"/>
-      <c r="AU144"/>
-      <c r="AV144"/>
-      <c r="AW144"/>
-      <c r="AX144"/>
-      <c r="AY144"/>
-      <c r="AZ144"/>
-      <c r="BA144"/>
-      <c r="BB144"/>
-      <c r="BC144"/>
-      <c r="BD144"/>
-      <c r="BE144"/>
-    </row>
-    <row r="145" spans="1:4" ht="15.75">
-      <c r="B145" s="9" t="s">
+      <c r="D143" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="144" spans="1:4" ht="15.75">
+      <c r="B144" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D144" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="145" spans="1:57" ht="15.75">
+      <c r="B145" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D145" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="146" spans="1:57" ht="15.75">
+      <c r="B146" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D146" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="147" spans="1:57" ht="15.75"/>
+    <row r="148" spans="1:57" ht="15.75">
+      <c r="A148" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B148" s="1"/>
+      <c r="C148" s="1"/>
+      <c r="D148" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="149" spans="1:57" ht="15.75">
+      <c r="A149" s="1"/>
+      <c r="B149" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="C149" s="1"/>
+      <c r="D149" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="150" spans="1:57" ht="15.75">
+      <c r="A150" s="50">
+        <f>SUM(E150:BE150)</f>
+        <v>0</v>
+      </c>
+      <c r="B150" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C145" s="9"/>
-      <c r="D145" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="146" spans="1:4" ht="15.75"/>
-    <row r="147" spans="1:4" ht="15.75"/>
-    <row r="148" spans="1:4" s="34" customFormat="1" ht="15.75">
-      <c r="A148" s="33" t="s">
+      <c r="D150" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="151" spans="1:57" ht="15.75">
+      <c r="B151" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D151" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="152" spans="1:57" ht="15.75">
+      <c r="B152" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D152" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="153" spans="1:57" ht="15.75">
+      <c r="B153" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D153" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="154" spans="1:57" ht="15.75"/>
+    <row r="155" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A155" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B155" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D155" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="156" spans="1:57" ht="15.75">
+      <c r="A156" s="50"/>
+      <c r="B156" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C156" s="9"/>
+      <c r="D156" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="157" spans="1:57" ht="15.75"/>
+    <row r="158" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A158" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D148" s="35"/>
-    </row>
-    <row r="149" spans="1:4" ht="15.75">
-      <c r="A149" s="1" t="s">
+      <c r="D158" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E158"/>
+      <c r="F158"/>
+      <c r="G158"/>
+      <c r="H158"/>
+      <c r="I158"/>
+      <c r="J158"/>
+      <c r="K158"/>
+      <c r="L158"/>
+      <c r="M158"/>
+      <c r="N158"/>
+      <c r="O158"/>
+      <c r="P158"/>
+      <c r="Q158"/>
+      <c r="R158"/>
+      <c r="S158"/>
+      <c r="T158"/>
+      <c r="U158"/>
+      <c r="V158"/>
+      <c r="W158"/>
+      <c r="X158"/>
+      <c r="Y158"/>
+      <c r="Z158"/>
+      <c r="AA158"/>
+      <c r="AB158"/>
+      <c r="AC158"/>
+      <c r="AD158"/>
+      <c r="AE158"/>
+      <c r="AF158"/>
+      <c r="AG158"/>
+      <c r="AH158"/>
+      <c r="AI158"/>
+      <c r="AJ158"/>
+      <c r="AK158"/>
+      <c r="AL158"/>
+      <c r="AM158"/>
+      <c r="AN158"/>
+      <c r="AO158"/>
+      <c r="AP158"/>
+      <c r="AQ158"/>
+      <c r="AR158"/>
+      <c r="AS158"/>
+      <c r="AT158"/>
+      <c r="AU158"/>
+      <c r="AV158"/>
+      <c r="AW158"/>
+      <c r="AX158"/>
+      <c r="AY158"/>
+      <c r="AZ158"/>
+      <c r="BA158"/>
+      <c r="BB158"/>
+      <c r="BC158"/>
+      <c r="BD158"/>
+      <c r="BE158"/>
+    </row>
+    <row r="159" spans="1:57" ht="15.75">
+      <c r="B159" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C159" s="9"/>
+      <c r="D159" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="160" spans="1:57" ht="15.75"/>
+    <row r="161" spans="1:4" ht="15.75"/>
+    <row r="162" spans="1:4" s="34" customFormat="1" ht="15.75">
+      <c r="A162" s="33" t="s">
+        <v>45</v>
+      </c>
+      <c r="D162" s="35"/>
+    </row>
+    <row r="163" spans="1:4" ht="15.75">
+      <c r="A163" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D149" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="150" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A150" s="3"/>
-      <c r="B150" s="4" t="s">
+      <c r="D163" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="164" spans="1:4" s="4" customFormat="1" ht="15.75">
+      <c r="A164" s="3"/>
+      <c r="B164" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D150" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="151" spans="1:4" s="7" customFormat="1" ht="15.75">
-      <c r="B151" s="7" t="s">
+      <c r="D164" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="165" spans="1:4" s="7" customFormat="1" ht="15.75">
+      <c r="B165" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D151" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="152" spans="1:4" s="7" customFormat="1" ht="15.75">
-      <c r="B152" s="7" t="s">
+      <c r="D165" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="166" spans="1:4" s="7" customFormat="1" ht="15.75">
+      <c r="B166" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C152" s="15"/>
-      <c r="D152" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="153" spans="1:4" s="9" customFormat="1" ht="15.75">
-      <c r="A153" s="50">
-        <f>SUM(E153:BE153)</f>
+      <c r="C166" s="15"/>
+      <c r="D166" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="167" spans="1:4" s="9" customFormat="1" ht="15.75">
+      <c r="A167" s="50">
+        <f>SUM(E167:BE167)</f>
         <v>0</v>
       </c>
-      <c r="B153" s="9" t="s">
+      <c r="B167" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D153" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="154" spans="1:4" ht="15.75"/>
-    <row r="155" spans="1:4" ht="15.75">
-      <c r="A155" s="1" t="s">
+      <c r="D167" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="168" spans="1:4" ht="15.75"/>
+    <row r="169" spans="1:4" ht="15.75">
+      <c r="A169" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D155" s="23" t="s">
+      <c r="D169" s="23" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="156" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A156" s="3"/>
-      <c r="B156" s="4" t="s">
+    <row r="170" spans="1:4" s="4" customFormat="1" ht="15.75">
+      <c r="A170" s="3"/>
+      <c r="B170" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D156" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="157" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A157" s="14"/>
-      <c r="B157" s="15" t="s">
+      <c r="D170" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A171" s="14"/>
+      <c r="B171" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D157" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="158" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A158" s="14"/>
-      <c r="B158" s="7" t="s">
+      <c r="D171" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="172" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A172" s="14"/>
+      <c r="B172" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D158" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="159" spans="1:4" s="12" customFormat="1" ht="15.75">
-      <c r="A159" s="50">
-        <f>SUM(E159:BE159)</f>
+      <c r="D172" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="173" spans="1:4" s="12" customFormat="1" ht="15.75">
+      <c r="A173" s="50">
+        <f>SUM(E173:BE173)</f>
         <v>0</v>
       </c>
-      <c r="B159" s="12" t="s">
+      <c r="B173" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D159" s="13" t="s">
+      <c r="D173" s="13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="15.75">
-      <c r="B160" t="s">
+    <row r="174" spans="1:4" ht="15.75">
+      <c r="B174" t="s">
         <v>15</v>
       </c>
-      <c r="C160" s="11" t="s">
+      <c r="C174" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D160" s="6" t="s">
+      <c r="D174" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="161" spans="1:57" ht="15.75">
-      <c r="C161" s="11" t="s">
+    <row r="175" spans="1:4" ht="15.75">
+      <c r="C175" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D161" s="6" t="s">
+      <c r="D175" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="162" spans="1:57" ht="15.75">
-      <c r="C162" s="6"/>
-    </row>
-    <row r="163" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A163" s="1" t="s">
+    <row r="176" spans="1:4" ht="15.75">
+      <c r="C176" s="6"/>
+    </row>
+    <row r="177" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A177" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B163" s="1" t="s">
+      <c r="B177" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D163" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="164" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="B164" s="1" t="s">
+      <c r="D177" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="178" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="B178" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D164" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="165" spans="1:57" s="9" customFormat="1" ht="15.75">
-      <c r="A165" s="50">
-        <f>SUM(E165:BE165)</f>
+      <c r="D178" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="179" spans="1:57" s="9" customFormat="1" ht="15.75">
+      <c r="A179" s="50">
+        <f>SUM(E179:BE179)</f>
         <v>0</v>
       </c>
-      <c r="B165" s="9" t="s">
+      <c r="B179" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="D165" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="166" spans="1:57" ht="15.75">
-      <c r="B166" s="7" t="s">
+      <c r="D179" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="180" spans="1:57" ht="15.75">
+      <c r="B180" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D166" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="167" spans="1:57" ht="15.75">
-      <c r="B167" s="7" t="s">
+      <c r="D180" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="181" spans="1:57" ht="15.75">
+      <c r="B181" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D167" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="168" spans="1:57" ht="15.75">
-      <c r="B168" s="7" t="s">
+      <c r="D181" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="182" spans="1:57" ht="15.75">
+      <c r="B182" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D168" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="169" spans="1:57" ht="15.75"/>
-    <row r="170" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A170" s="1" t="s">
+      <c r="D182" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="183" spans="1:57" ht="15.75"/>
+    <row r="184" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A184" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D170" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E170"/>
-      <c r="F170"/>
-      <c r="G170"/>
-      <c r="H170"/>
-      <c r="I170"/>
-      <c r="J170"/>
-      <c r="K170"/>
-      <c r="L170"/>
-      <c r="M170"/>
-      <c r="N170"/>
-      <c r="O170"/>
-      <c r="P170"/>
-      <c r="Q170"/>
-      <c r="R170"/>
-      <c r="S170"/>
-      <c r="T170"/>
-      <c r="U170"/>
-      <c r="V170"/>
-      <c r="W170"/>
-      <c r="X170"/>
-      <c r="Y170"/>
-      <c r="Z170"/>
-      <c r="AA170"/>
-      <c r="AB170"/>
-      <c r="AC170"/>
-      <c r="AD170"/>
-      <c r="AE170"/>
-      <c r="AF170"/>
-      <c r="AG170"/>
-      <c r="AH170"/>
-      <c r="AI170"/>
-      <c r="AJ170"/>
-      <c r="AK170"/>
-      <c r="AL170"/>
-      <c r="AM170"/>
-      <c r="AN170"/>
-      <c r="AO170"/>
-      <c r="AP170"/>
-      <c r="AQ170"/>
-      <c r="AR170"/>
-      <c r="AS170"/>
-      <c r="AT170"/>
-      <c r="AU170"/>
-      <c r="AV170"/>
-      <c r="AW170"/>
-      <c r="AX170"/>
-      <c r="AY170"/>
-      <c r="AZ170"/>
-      <c r="BA170"/>
-      <c r="BB170"/>
-      <c r="BC170"/>
-      <c r="BD170"/>
-      <c r="BE170"/>
-    </row>
-    <row r="171" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="B171" s="1" t="s">
+      <c r="D184" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E184"/>
+      <c r="F184"/>
+      <c r="G184"/>
+      <c r="H184"/>
+      <c r="I184"/>
+      <c r="J184"/>
+      <c r="K184"/>
+      <c r="L184"/>
+      <c r="M184"/>
+      <c r="N184"/>
+      <c r="O184"/>
+      <c r="P184"/>
+      <c r="Q184"/>
+      <c r="R184"/>
+      <c r="S184"/>
+      <c r="T184"/>
+      <c r="U184"/>
+      <c r="V184"/>
+      <c r="W184"/>
+      <c r="X184"/>
+      <c r="Y184"/>
+      <c r="Z184"/>
+      <c r="AA184"/>
+      <c r="AB184"/>
+      <c r="AC184"/>
+      <c r="AD184"/>
+      <c r="AE184"/>
+      <c r="AF184"/>
+      <c r="AG184"/>
+      <c r="AH184"/>
+      <c r="AI184"/>
+      <c r="AJ184"/>
+      <c r="AK184"/>
+      <c r="AL184"/>
+      <c r="AM184"/>
+      <c r="AN184"/>
+      <c r="AO184"/>
+      <c r="AP184"/>
+      <c r="AQ184"/>
+      <c r="AR184"/>
+      <c r="AS184"/>
+      <c r="AT184"/>
+      <c r="AU184"/>
+      <c r="AV184"/>
+      <c r="AW184"/>
+      <c r="AX184"/>
+      <c r="AY184"/>
+      <c r="AZ184"/>
+      <c r="BA184"/>
+      <c r="BB184"/>
+      <c r="BC184"/>
+      <c r="BD184"/>
+      <c r="BE184"/>
+    </row>
+    <row r="185" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="B185" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D171" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E171"/>
-      <c r="F171"/>
-      <c r="G171"/>
-      <c r="H171"/>
-      <c r="I171"/>
-      <c r="J171"/>
-      <c r="K171"/>
-      <c r="L171"/>
-      <c r="M171"/>
-      <c r="N171"/>
-      <c r="O171"/>
-      <c r="P171"/>
-      <c r="Q171"/>
-      <c r="R171"/>
-      <c r="S171"/>
-      <c r="T171"/>
-      <c r="U171"/>
-      <c r="V171"/>
-      <c r="W171"/>
-      <c r="X171"/>
-      <c r="Y171"/>
-      <c r="Z171"/>
-      <c r="AA171"/>
-      <c r="AB171"/>
-      <c r="AC171"/>
-      <c r="AD171"/>
-      <c r="AE171"/>
-      <c r="AF171"/>
-      <c r="AG171"/>
-      <c r="AH171"/>
-      <c r="AI171"/>
-      <c r="AJ171"/>
-      <c r="AK171"/>
-      <c r="AL171"/>
-      <c r="AM171"/>
-      <c r="AN171"/>
-      <c r="AO171"/>
-      <c r="AP171"/>
-      <c r="AQ171"/>
-      <c r="AR171"/>
-      <c r="AS171"/>
-      <c r="AT171"/>
-      <c r="AU171"/>
-      <c r="AV171"/>
-      <c r="AW171"/>
-      <c r="AX171"/>
-      <c r="AY171"/>
-      <c r="AZ171"/>
-      <c r="BA171"/>
-      <c r="BB171"/>
-      <c r="BC171"/>
-      <c r="BD171"/>
-      <c r="BE171"/>
-    </row>
-    <row r="172" spans="1:57" ht="15.75">
-      <c r="A172" s="50">
-        <f>SUM(E172:BE172)</f>
+      <c r="D185" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E185"/>
+      <c r="F185"/>
+      <c r="G185"/>
+      <c r="H185"/>
+      <c r="I185"/>
+      <c r="J185"/>
+      <c r="K185"/>
+      <c r="L185"/>
+      <c r="M185"/>
+      <c r="N185"/>
+      <c r="O185"/>
+      <c r="P185"/>
+      <c r="Q185"/>
+      <c r="R185"/>
+      <c r="S185"/>
+      <c r="T185"/>
+      <c r="U185"/>
+      <c r="V185"/>
+      <c r="W185"/>
+      <c r="X185"/>
+      <c r="Y185"/>
+      <c r="Z185"/>
+      <c r="AA185"/>
+      <c r="AB185"/>
+      <c r="AC185"/>
+      <c r="AD185"/>
+      <c r="AE185"/>
+      <c r="AF185"/>
+      <c r="AG185"/>
+      <c r="AH185"/>
+      <c r="AI185"/>
+      <c r="AJ185"/>
+      <c r="AK185"/>
+      <c r="AL185"/>
+      <c r="AM185"/>
+      <c r="AN185"/>
+      <c r="AO185"/>
+      <c r="AP185"/>
+      <c r="AQ185"/>
+      <c r="AR185"/>
+      <c r="AS185"/>
+      <c r="AT185"/>
+      <c r="AU185"/>
+      <c r="AV185"/>
+      <c r="AW185"/>
+      <c r="AX185"/>
+      <c r="AY185"/>
+      <c r="AZ185"/>
+      <c r="BA185"/>
+      <c r="BB185"/>
+      <c r="BC185"/>
+      <c r="BD185"/>
+      <c r="BE185"/>
+    </row>
+    <row r="186" spans="1:57" ht="15.75">
+      <c r="A186" s="50">
+        <f>SUM(E186:BE186)</f>
         <v>0</v>
       </c>
-      <c r="B172" s="9" t="s">
+      <c r="B186" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C172" s="9"/>
-      <c r="D172" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="173" spans="1:57" ht="15.75">
-      <c r="B173" s="7" t="s">
+      <c r="C186" s="9"/>
+      <c r="D186" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="187" spans="1:57" ht="15.75">
+      <c r="B187" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="D173" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="174" spans="1:57" ht="15.75">
-      <c r="B174" s="7" t="s">
+      <c r="D187" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="188" spans="1:57" ht="15.75">
+      <c r="B188" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D174" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="175" spans="1:57" ht="15.75">
-      <c r="B175" s="7" t="s">
+      <c r="D188" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="189" spans="1:57" ht="15.75">
+      <c r="B189" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D175" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="176" spans="1:57" ht="15.75"/>
-    <row r="177" spans="1:4" ht="15.75"/>
-    <row r="178" spans="1:4" s="37" customFormat="1" ht="15.75">
-      <c r="A178" s="36" t="s">
-        <v>44</v>
-      </c>
-      <c r="D178" s="38"/>
-    </row>
-    <row r="179" spans="1:4" ht="15.75">
-      <c r="A179" s="1" t="s">
+      <c r="D189" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="190" spans="1:57" ht="15.75"/>
+    <row r="191" spans="1:57" ht="15.75"/>
+    <row r="192" spans="1:57" s="37" customFormat="1" ht="15.75">
+      <c r="A192" s="36" t="s">
+        <v>46</v>
+      </c>
+      <c r="D192" s="38"/>
+    </row>
+    <row r="193" spans="1:4" ht="15.75">
+      <c r="A193" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D179" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="180" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A180" s="3"/>
-      <c r="B180" s="4" t="s">
+      <c r="D193" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="194" spans="1:4" s="4" customFormat="1" ht="15.75">
+      <c r="A194" s="3"/>
+      <c r="B194" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D180" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="181" spans="1:4" s="7" customFormat="1" ht="15.75">
-      <c r="B181" s="7" t="s">
+      <c r="D194" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="195" spans="1:4" s="7" customFormat="1" ht="15.75">
+      <c r="B195" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D181" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="182" spans="1:4" s="7" customFormat="1" ht="15.75">
-      <c r="B182" s="7" t="s">
+      <c r="D195" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="196" spans="1:4" s="7" customFormat="1" ht="15.75">
+      <c r="B196" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C182" s="15"/>
-      <c r="D182" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="183" spans="1:4" s="9" customFormat="1" ht="15.75">
-      <c r="A183" s="50">
-        <f>SUM(E183:BE183)</f>
+      <c r="C196" s="15"/>
+      <c r="D196" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="197" spans="1:4" s="9" customFormat="1" ht="15.75">
+      <c r="A197" s="50">
+        <f>SUM(E197:BE197)</f>
         <v>0</v>
       </c>
-      <c r="B183" s="9" t="s">
+      <c r="B197" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D183" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="184" spans="1:4" ht="15.75"/>
-    <row r="185" spans="1:4" ht="15.75">
-      <c r="A185" s="1" t="s">
+      <c r="D197" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="198" spans="1:4" ht="15.75"/>
+    <row r="199" spans="1:4" ht="15.75">
+      <c r="A199" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="D185" s="23" t="s">
+      <c r="D199" s="23" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="186" spans="1:4" s="4" customFormat="1" ht="15.75">
-      <c r="A186" s="3"/>
-      <c r="B186" s="4" t="s">
+    <row r="200" spans="1:4" s="4" customFormat="1" ht="15.75">
+      <c r="A200" s="3"/>
+      <c r="B200" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D186" s="32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="187" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A187" s="14"/>
-      <c r="B187" s="15" t="s">
+      <c r="D200" s="32" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="201" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A201" s="14"/>
+      <c r="B201" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="D187" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" s="15" customFormat="1" ht="15.75">
-      <c r="A188" s="14"/>
-      <c r="B188" s="7" t="s">
+      <c r="D201" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="202" spans="1:4" s="15" customFormat="1" ht="15.75">
+      <c r="A202" s="14"/>
+      <c r="B202" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D188" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="189" spans="1:4" s="12" customFormat="1" ht="15.75">
-      <c r="A189" s="50">
-        <f>SUM(E189:BE189)</f>
+      <c r="D202" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="203" spans="1:4" s="12" customFormat="1" ht="15.75">
+      <c r="A203" s="50">
+        <f>SUM(E203:BE203)</f>
         <v>0</v>
       </c>
-      <c r="B189" s="12" t="s">
+      <c r="B203" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="D189" s="13" t="s">
+      <c r="D203" s="13" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="190" spans="1:4" ht="15.75">
-      <c r="B190" t="s">
+    <row r="204" spans="1:4" ht="15.75">
+      <c r="B204" t="s">
         <v>15</v>
       </c>
-      <c r="C190" s="11" t="s">
+      <c r="C204" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D190" s="6" t="s">
+      <c r="D204" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="191" spans="1:4" ht="15.75">
-      <c r="C191" s="11" t="s">
+    <row r="205" spans="1:4" ht="15.75">
+      <c r="C205" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="D191" s="6" t="s">
+      <c r="D205" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="192" spans="1:4" ht="15.75">
-      <c r="C192" s="6"/>
-    </row>
-    <row r="193" spans="1:4" s="1" customFormat="1" ht="15.75">
-      <c r="A193" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B193" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D193" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="194" spans="1:4" s="1" customFormat="1" ht="15.75">
-      <c r="B194" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="D194" s="31" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="195" spans="1:4" s="9" customFormat="1" ht="15.75">
-      <c r="A195" s="50">
-        <f>SUM(E195:BE195)</f>
-        <v>0</v>
-      </c>
-      <c r="B195" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="D195" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="196" spans="1:4" ht="15.75">
-      <c r="B196" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D196" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="197" spans="1:4" ht="15.75">
-      <c r="B197" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D197" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="198" spans="1:4" ht="15.75">
-      <c r="B198" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D198" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="199" spans="1:4" ht="15.75"/>
-    <row r="200" spans="1:4" ht="15.75">
-      <c r="A200" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B200" s="1"/>
-      <c r="C200" s="1"/>
-      <c r="D200" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="201" spans="1:4" ht="15.75">
-      <c r="A201" s="1"/>
-      <c r="B201" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C201" s="1"/>
-      <c r="D201" s="23" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="202" spans="1:4" ht="15.75">
-      <c r="A202" s="50">
-        <f>SUM(E202:BE202)</f>
-        <v>0</v>
-      </c>
-      <c r="B202" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="C202" s="9"/>
-      <c r="D202" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="203" spans="1:4" ht="15.75">
-      <c r="B203" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D203" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="204" spans="1:4" ht="15.75">
-      <c r="B204" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D204" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="205" spans="1:4" ht="15.75">
-      <c r="B205" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="D205" s="16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="206" spans="1:4" ht="15.75"/>
+    <row r="206" spans="1:4" ht="15.75">
+      <c r="C206" s="6"/>
+    </row>
     <row r="207" spans="1:4" s="1" customFormat="1" ht="15.75">
       <c r="A207" s="1" t="s">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="B207" s="1" t="s">
         <v>26</v>
@@ -3047,130 +3053,244 @@
         <v>3</v>
       </c>
     </row>
-    <row r="208" spans="1:4" ht="15.75">
-      <c r="B208" s="9" t="s">
+    <row r="208" spans="1:4" s="1" customFormat="1" ht="15.75">
+      <c r="B208" s="48" t="s">
+        <v>27</v>
+      </c>
+      <c r="D208" s="31" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="209" spans="1:57" s="9" customFormat="1" ht="15.75">
+      <c r="A209" s="50">
+        <f>SUM(E209:BE209)</f>
+        <v>0</v>
+      </c>
+      <c r="B209" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C208" s="9"/>
-      <c r="D208" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="209" spans="1:57" ht="15.75"/>
-    <row r="210" spans="1:57" s="1" customFormat="1" ht="15.75">
-      <c r="A210" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D210" s="23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E210"/>
-      <c r="F210"/>
-      <c r="G210"/>
-      <c r="H210"/>
-      <c r="I210"/>
-      <c r="J210"/>
-      <c r="K210"/>
-      <c r="L210"/>
-      <c r="M210"/>
-      <c r="N210"/>
-      <c r="O210"/>
-      <c r="P210"/>
-      <c r="Q210"/>
-      <c r="R210"/>
-      <c r="S210"/>
-      <c r="T210"/>
-      <c r="U210"/>
-      <c r="V210"/>
-      <c r="W210"/>
-      <c r="X210"/>
-      <c r="Y210"/>
-      <c r="Z210"/>
-      <c r="AA210"/>
-      <c r="AB210"/>
-      <c r="AC210"/>
-      <c r="AD210"/>
-      <c r="AE210"/>
-      <c r="AF210"/>
-      <c r="AG210"/>
-      <c r="AH210"/>
-      <c r="AI210"/>
-      <c r="AJ210"/>
-      <c r="AK210"/>
-      <c r="AL210"/>
-      <c r="AM210"/>
-      <c r="AN210"/>
-      <c r="AO210"/>
-      <c r="AP210"/>
-      <c r="AQ210"/>
-      <c r="AR210"/>
-      <c r="AS210"/>
-      <c r="AT210"/>
-      <c r="AU210"/>
-      <c r="AV210"/>
-      <c r="AW210"/>
-      <c r="AX210"/>
-      <c r="AY210"/>
-      <c r="AZ210"/>
-      <c r="BA210"/>
-      <c r="BB210"/>
-      <c r="BC210"/>
-      <c r="BD210"/>
-      <c r="BE210"/>
+      <c r="D209" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="210" spans="1:57" ht="15.75">
+      <c r="B210" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D210" s="16" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="211" spans="1:57" ht="15.75">
-      <c r="B211" s="9" t="s">
+      <c r="B211" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D211" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="212" spans="1:57" ht="15.75">
+      <c r="B212" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D212" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="213" spans="1:57" ht="15.75"/>
+    <row r="214" spans="1:57" ht="15.75">
+      <c r="A214" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B214" s="1"/>
+      <c r="C214" s="1"/>
+      <c r="D214" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="215" spans="1:57" ht="15.75">
+      <c r="A215" s="1"/>
+      <c r="B215" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C215" s="1"/>
+      <c r="D215" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="216" spans="1:57" ht="15.75">
+      <c r="A216" s="50">
+        <f>SUM(E216:BE216)</f>
+        <v>0</v>
+      </c>
+      <c r="B216" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C211" s="9"/>
-      <c r="D211" s="10" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="212" spans="1:57" ht="15.75"/>
-    <row r="213" spans="1:57" ht="15.75"/>
-    <row r="214" spans="1:57" ht="15.75"/>
-    <row r="215" spans="1:57" ht="15.75"/>
-    <row r="216" spans="1:57" ht="15.75"/>
-    <row r="217" spans="1:57" ht="15.75"/>
-    <row r="218" spans="1:57" ht="15.75"/>
-    <row r="219" spans="1:57" ht="15.75"/>
+      <c r="C216" s="9"/>
+      <c r="D216" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="217" spans="1:57" ht="15.75">
+      <c r="B217" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D217" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="218" spans="1:57" ht="15.75">
+      <c r="B218" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="D218" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="219" spans="1:57" ht="15.75">
+      <c r="B219" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D219" s="16" t="s">
+        <v>11</v>
+      </c>
+    </row>
     <row r="220" spans="1:57" ht="15.75"/>
-    <row r="221" spans="1:57" ht="15.75"/>
-    <row r="222" spans="1:57" ht="15.75"/>
+    <row r="221" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A221" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B221" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D221" s="23" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="222" spans="1:57" ht="15.75">
+      <c r="B222" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C222" s="9"/>
+      <c r="D222" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
     <row r="223" spans="1:57" ht="15.75"/>
-    <row r="224" spans="1:57" ht="15.75"/>
-    <row r="225" ht="15.75"/>
-    <row r="226" ht="15.75"/>
-    <row r="227" ht="15.75"/>
-    <row r="228" ht="15.75"/>
-    <row r="229" ht="15.75"/>
-    <row r="230" ht="15.75"/>
-    <row r="231" ht="15.75"/>
-    <row r="232" ht="15.75"/>
-    <row r="233" ht="15.75"/>
-    <row r="234" ht="15.75"/>
-    <row r="235" ht="15.75"/>
-    <row r="236" ht="15.75"/>
-    <row r="237" ht="15.75"/>
-    <row r="238" ht="15.75"/>
-    <row r="239" ht="15.75"/>
-    <row r="240" ht="15.75"/>
-    <row r="241" spans="4:4" ht="15.75"/>
-    <row r="242" spans="4:4" ht="15.75"/>
-    <row r="243" spans="4:4" ht="15.75"/>
-    <row r="244" spans="4:4" ht="15.75"/>
-    <row r="245" spans="4:4" ht="15.75">
-      <c r="D245"/>
-    </row>
-    <row r="246" spans="4:4" ht="15.75">
-      <c r="D246"/>
-    </row>
-    <row r="247" spans="4:4" ht="15.75">
-      <c r="D247"/>
-    </row>
-    <row r="248" spans="4:4" ht="15.75">
-      <c r="D248"/>
+    <row r="224" spans="1:57" s="1" customFormat="1" ht="15.75">
+      <c r="A224" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D224" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="E224"/>
+      <c r="F224"/>
+      <c r="G224"/>
+      <c r="H224"/>
+      <c r="I224"/>
+      <c r="J224"/>
+      <c r="K224"/>
+      <c r="L224"/>
+      <c r="M224"/>
+      <c r="N224"/>
+      <c r="O224"/>
+      <c r="P224"/>
+      <c r="Q224"/>
+      <c r="R224"/>
+      <c r="S224"/>
+      <c r="T224"/>
+      <c r="U224"/>
+      <c r="V224"/>
+      <c r="W224"/>
+      <c r="X224"/>
+      <c r="Y224"/>
+      <c r="Z224"/>
+      <c r="AA224"/>
+      <c r="AB224"/>
+      <c r="AC224"/>
+      <c r="AD224"/>
+      <c r="AE224"/>
+      <c r="AF224"/>
+      <c r="AG224"/>
+      <c r="AH224"/>
+      <c r="AI224"/>
+      <c r="AJ224"/>
+      <c r="AK224"/>
+      <c r="AL224"/>
+      <c r="AM224"/>
+      <c r="AN224"/>
+      <c r="AO224"/>
+      <c r="AP224"/>
+      <c r="AQ224"/>
+      <c r="AR224"/>
+      <c r="AS224"/>
+      <c r="AT224"/>
+      <c r="AU224"/>
+      <c r="AV224"/>
+      <c r="AW224"/>
+      <c r="AX224"/>
+      <c r="AY224"/>
+      <c r="AZ224"/>
+      <c r="BA224"/>
+      <c r="BB224"/>
+      <c r="BC224"/>
+      <c r="BD224"/>
+      <c r="BE224"/>
+    </row>
+    <row r="225" spans="2:4" ht="15.75">
+      <c r="B225" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C225" s="9"/>
+      <c r="D225" s="10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="226" spans="2:4" ht="15.75"/>
+    <row r="227" spans="2:4" ht="15.75"/>
+    <row r="228" spans="2:4" ht="15.75"/>
+    <row r="229" spans="2:4" ht="15.75"/>
+    <row r="230" spans="2:4" ht="15.75"/>
+    <row r="231" spans="2:4" ht="15.75"/>
+    <row r="232" spans="2:4" ht="15.75"/>
+    <row r="233" spans="2:4" ht="15.75"/>
+    <row r="234" spans="2:4" ht="15.75"/>
+    <row r="235" spans="2:4" ht="15.75"/>
+    <row r="236" spans="2:4" ht="15.75"/>
+    <row r="237" spans="2:4" ht="15.75"/>
+    <row r="238" spans="2:4" ht="15.75"/>
+    <row r="239" spans="2:4" ht="15.75"/>
+    <row r="240" spans="2:4" ht="15.75"/>
+    <row r="241" ht="15.75"/>
+    <row r="242" ht="15.75"/>
+    <row r="243" ht="15.75"/>
+    <row r="244" ht="15.75"/>
+    <row r="245" ht="15.75"/>
+    <row r="246" ht="15.75"/>
+    <row r="247" ht="15.75"/>
+    <row r="248" ht="15.75"/>
+    <row r="249" ht="15.75"/>
+    <row r="250" ht="15.75"/>
+    <row r="251" ht="15.75"/>
+    <row r="252" ht="15.75"/>
+    <row r="253" ht="15.75"/>
+    <row r="254" ht="15.75"/>
+    <row r="255" ht="15.75"/>
+    <row r="256" ht="15.75"/>
+    <row r="257" spans="4:4" ht="15.75"/>
+    <row r="258" spans="4:4" ht="15.75"/>
+    <row r="259" spans="4:4" ht="15.75">
+      <c r="D259"/>
+    </row>
+    <row r="260" spans="4:4" ht="15.75">
+      <c r="D260"/>
+    </row>
+    <row r="261" spans="4:4" ht="15.75">
+      <c r="D261"/>
+    </row>
+    <row r="262" spans="4:4" ht="15.75">
+      <c r="D262"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>